<commit_message>
Approve 200 reviewed editorial ideas for planning v1.10.1
</commit_message>
<xml_diff>
--- a/communication/research/HSF_Knowledge_Data_Insight_260_Idea_Bank_Editorial_Inventory.xlsx
+++ b/communication/research/HSF_Knowledge_Data_Insight_260_Idea_Bank_Editorial_Inventory.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re46612cab2a14405"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas" sheetId="2" r:id="R445b8a9c15ab4abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial Rules" sheetId="3" r:id="R269f0e8104974201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0b12e59c9c4d4904"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas" sheetId="2" r:id="Re80b8548a0114e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial Rules" sheetId="3" r:id="R650b248b22924516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval History" sheetId="4" r:id="R67d9dd90da7741f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -38,13 +39,28 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF006B35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF8F3"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -64,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -95,6 +111,11 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -327,7 +348,7 @@
   <x:sheetData>
     <x:row r="1" ht="31" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>HSF KDI Editorial Idea Inventory — v1.9.0</x:v>
+        <x:v>HSF KDI Editorial Idea Inventory — v1.10.1</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str"/>
       <x:c r="C1" s="3" t="str"/>
@@ -356,15 +377,15 @@
         <x:v>Editorial approved</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>160</x:v>
+        <x:v>260</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="str">
-        <x:v>New proposed</x:v>
+        <x:v>Editorial proposed (remaining)</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>100</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -403,7 +424,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
-        <x:v>KDI-161..260 are proposed; KDI-135..160 and PSC-121..140 were promoted on 2026-10-30 by user direction.</x:v>
+        <x:v>KDI-161..260 approved for editorial planning on 2026-10-30 by user review. Original source leads and factual claims remain unverified; exact post approval remains separate.</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str"/>
       <x:c r="C12" s="10" t="str"/>
@@ -7749,7 +7770,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K162" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L162" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -7799,7 +7820,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K163" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L163" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -7849,7 +7870,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K164" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L164" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -7899,7 +7920,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K165" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L165" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -7949,7 +7970,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K166" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L166" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -7999,7 +8020,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K167" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L167" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8049,7 +8070,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K168" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L168" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8099,7 +8120,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K169" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L169" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8149,7 +8170,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K170" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L170" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8199,7 +8220,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K171" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L171" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8249,7 +8270,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K172" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L172" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8299,7 +8320,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K173" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L173" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8349,7 +8370,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K174" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L174" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8399,7 +8420,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K175" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L175" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8449,7 +8470,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K176" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L176" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8499,7 +8520,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K177" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L177" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8549,7 +8570,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K178" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L178" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8599,7 +8620,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K179" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L179" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8649,7 +8670,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K180" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L180" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8699,7 +8720,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K181" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L181" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8749,7 +8770,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K182" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L182" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8799,7 +8820,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K183" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L183" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8849,7 +8870,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K184" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L184" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8899,7 +8920,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K185" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L185" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8949,7 +8970,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K186" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L186" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -8999,7 +9020,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K187" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L187" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9049,7 +9070,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K188" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L188" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9099,7 +9120,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K189" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L189" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9149,7 +9170,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K190" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L190" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9199,7 +9220,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K191" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L191" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9249,7 +9270,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K192" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L192" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9299,7 +9320,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K193" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L193" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9349,7 +9370,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K194" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L194" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9399,7 +9420,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K195" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L195" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9449,7 +9470,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K196" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L196" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9499,7 +9520,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K197" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L197" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9549,7 +9570,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K198" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L198" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9599,7 +9620,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K199" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L199" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9649,7 +9670,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K200" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L200" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9699,7 +9720,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K201" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L201" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9749,7 +9770,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K202" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L202" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9799,7 +9820,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K203" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L203" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9849,7 +9870,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K204" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L204" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9899,7 +9920,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K205" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L205" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9949,7 +9970,7 @@
         <x:v>Climate science and policy source review; distinguish proposals, observations, projections and published commitments; validate date, uncertainty and Bangladesh context.</x:v>
       </x:c>
       <x:c r="K206" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L206" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -9999,7 +10020,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K207" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L207" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10049,7 +10070,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K208" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L208" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10099,7 +10120,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K209" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L209" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10149,7 +10170,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K210" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L210" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10199,7 +10220,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K211" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L211" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10249,7 +10270,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K212" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L212" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10299,7 +10320,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K213" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L213" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10349,7 +10370,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K214" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L214" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10399,7 +10420,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K215" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L215" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10449,7 +10470,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K216" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L216" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10499,7 +10520,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K217" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L217" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10549,7 +10570,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K218" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L218" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10599,7 +10620,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K219" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L219" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10649,7 +10670,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K220" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L220" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10699,7 +10720,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K221" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L221" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10749,7 +10770,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K222" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L222" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10799,7 +10820,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K223" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L223" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10849,7 +10870,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K224" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L224" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10899,7 +10920,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K225" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L225" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10949,7 +10970,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K226" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L226" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -10999,7 +11020,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K227" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L227" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11049,7 +11070,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K228" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L228" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11099,7 +11120,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K229" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L229" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11149,7 +11170,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K230" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L230" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11199,7 +11220,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K231" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L231" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11249,7 +11270,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K232" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L232" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11299,7 +11320,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K233" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L233" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11349,7 +11370,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K234" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L234" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11399,7 +11420,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K235" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L235" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11449,7 +11470,7 @@
         <x:v>Education pedagogy reviewer, inclusive-language and child safeguards; original learning-science source and Bangladesh applicability.</x:v>
       </x:c>
       <x:c r="K236" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L236" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11499,7 +11520,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K237" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L237" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11549,7 +11570,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K238" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L238" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11599,7 +11620,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K239" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L239" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11649,7 +11670,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K240" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L240" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11699,7 +11720,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K241" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L241" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11749,7 +11770,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K242" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L242" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11799,7 +11820,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K243" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L243" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11849,7 +11870,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K244" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L244" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11899,7 +11920,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K245" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L245" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11949,7 +11970,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K246" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L246" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -11999,7 +12020,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K247" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L247" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12049,7 +12070,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K248" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L248" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12099,7 +12120,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K249" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L249" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12149,7 +12170,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K250" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L250" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12199,7 +12220,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K251" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L251" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12249,7 +12270,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K252" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L252" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12299,7 +12320,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K253" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L253" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12349,7 +12370,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K254" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L254" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12399,7 +12420,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K255" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L255" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12449,7 +12470,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K256" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L256" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12499,7 +12520,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K257" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L257" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12549,7 +12570,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K258" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L258" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12599,7 +12620,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K259" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L259" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12649,7 +12670,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K260" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L260" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12699,7 +12720,7 @@
         <x:v>Licensed clinician and national/local guideline check; no medical diagnosis or individualized instructions; source/date/clinical safeguarding.</x:v>
       </x:c>
       <x:c r="K261" s="16" t="str">
-        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
       </x:c>
       <x:c r="L261" s="16" t="str">
         <x:v>NOT_VERIFIED</x:v>
@@ -12720,7 +12741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62674a977f894937"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69df0994be464a44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12808,4 +12829,71 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="27" customHeight="1">
+      <x:c r="A1" s="20" t="str">
+        <x:v>KDI 100-IDEA APPROVAL TRANSITION</x:v>
+      </x:c>
+      <x:c r="B1" s="20"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="22" t="str">
+        <x:v>Approval scope</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="str">
+        <x:v>Editorial planning ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="22" t="str">
+        <x:v>Idea IDs</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>KDI-161 through KDI-260</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="22" t="str">
+        <x:v>Prior status</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>EDITORIAL_IDEA_PROPOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="str">
+        <x:v>Current status</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>EDITORIAL_IDEA_APPROVED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="str">
+        <x:v>Review record</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>governance/EDITORIAL_APPROVAL_TRANSITION_v1.10.1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="str">
+        <x:v>Publication status</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>NOT_APPROVED — evidence and authorized final output review required</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>